<commit_message>
Added experiments and reevaluated growth stat testing
</commit_message>
<xml_diff>
--- a/data/compound_library/library.xlsx
+++ b/data/compound_library/library.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10119"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10420"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://chalmers-my.sharepoint.com/personal/danbru_chalmers_se/Documents/Desktop/GenExp/data/compound_library/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/danbru/Library/CloudStorage/OneDrive-Chalmers/Desktop/GenExp/data/compound_library/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="153" documentId="8_{45E8D5E7-04FD-CB42-BA2A-031D6C014692}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{92EDA852-4B4E-2F44-9DCD-09099A035242}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B706F176-FAFC-5E4A-A858-9609A912B726}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38400" yWindow="-8840" windowWidth="21600" windowHeight="37900" xr2:uid="{5207ED13-6406-E44B-8029-6CEF5067A94D}"/>
+    <workbookView xWindow="-35840" yWindow="500" windowWidth="35840" windowHeight="21900" xr2:uid="{5207ED13-6406-E44B-8029-6CEF5067A94D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" concurrentCalc="0"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="46">
   <si>
     <t>Compound</t>
   </si>
@@ -137,7 +137,43 @@
     <t>1% (v/v)</t>
   </si>
   <si>
-    <t>Chitosan</t>
+    <t>L-Glutamine</t>
+  </si>
+  <si>
+    <t>ZDXPYRJPNDTMRX-VKHMYHEASA-N</t>
+  </si>
+  <si>
+    <t>Acetic acid</t>
+  </si>
+  <si>
+    <t>50mM</t>
+  </si>
+  <si>
+    <t>250mM</t>
+  </si>
+  <si>
+    <t>500mM</t>
+  </si>
+  <si>
+    <t>QTBSBXVTEAMEQO-UHFFFAOYSA-N</t>
+  </si>
+  <si>
+    <t>25mM</t>
+  </si>
+  <si>
+    <t>100mM</t>
+  </si>
+  <si>
+    <t>L-Threonine</t>
+  </si>
+  <si>
+    <t>L-Lysine</t>
+  </si>
+  <si>
+    <t>KDXKERNSBIXSRK-YFKPBYRVSA-N</t>
+  </si>
+  <si>
+    <t>AYFVYJQAPQTCCC-GBXIJSLDSA-N</t>
   </si>
 </sst>
 </file>
@@ -242,10 +278,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -565,7 +597,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C37B54C-13B4-4F49-B23D-63B14E507B7A}">
-  <dimension ref="A1:C37"/>
+  <dimension ref="A1:C42"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="28.33203125" customWidth="1"/>
@@ -592,7 +624,7 @@
         <v>22</v>
       </c>
       <c r="C2" t="s">
-        <v>25</v>
+        <v>14</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
@@ -603,29 +635,29 @@
         <v>22</v>
       </c>
       <c r="C3" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="C4" t="s">
-        <v>14</v>
+        <v>25</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="C5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
@@ -636,7 +668,7 @@
         <v>8</v>
       </c>
       <c r="C6" t="s">
-        <v>25</v>
+        <v>14</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
@@ -647,29 +679,29 @@
         <v>8</v>
       </c>
       <c r="C7" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C8" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C9" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.2">
@@ -680,7 +712,7 @@
         <v>7</v>
       </c>
       <c r="C10" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.2">
@@ -691,7 +723,7 @@
         <v>7</v>
       </c>
       <c r="C11" t="s">
-        <v>25</v>
+        <v>14</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.2">
@@ -702,29 +734,29 @@
         <v>7</v>
       </c>
       <c r="C12" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C13" t="s">
-        <v>14</v>
+        <v>25</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C14" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.2">
@@ -735,7 +767,7 @@
         <v>10</v>
       </c>
       <c r="C15" t="s">
-        <v>25</v>
+        <v>14</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.2">
@@ -746,29 +778,29 @@
         <v>10</v>
       </c>
       <c r="C16" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="C17" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="C18" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.2">
@@ -779,187 +811,260 @@
         <v>23</v>
       </c>
       <c r="C19" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C20" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C21" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="C22" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="C23" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="C24" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>11</v>
+        <v>28</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>12</v>
+        <v>29</v>
       </c>
       <c r="C25" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C26" t="s">
-        <v>25</v>
+        <v>14</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>26</v>
-      </c>
-      <c r="B27" s="2" t="s">
-        <v>27</v>
+        <v>31</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>30</v>
       </c>
       <c r="C27" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>26</v>
-      </c>
-      <c r="B28" s="2" t="s">
-        <v>27</v>
+        <v>31</v>
+      </c>
+      <c r="B28" s="4" t="s">
+        <v>30</v>
       </c>
       <c r="C28" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>26</v>
-      </c>
-      <c r="B29" s="2" t="s">
-        <v>27</v>
+        <v>31</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>30</v>
       </c>
       <c r="C29" t="s">
-        <v>15</v>
+        <v>32</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="C30" t="s">
-        <v>13</v>
+        <v>25</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="C31" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>31</v>
-      </c>
-      <c r="B32" s="4" t="s">
-        <v>30</v>
+        <v>33</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>34</v>
       </c>
       <c r="C32" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>31</v>
-      </c>
-      <c r="B33" s="4" t="s">
-        <v>30</v>
+        <v>33</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>34</v>
       </c>
       <c r="C33" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>31</v>
-      </c>
-      <c r="B34" s="4" t="s">
-        <v>30</v>
+        <v>35</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>39</v>
       </c>
       <c r="C34" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>33</v>
+        <v>35</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C35" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>33</v>
+        <v>35</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C36" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>33</v>
+        <v>42</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C37" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A38" t="s">
+        <v>42</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C38" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A39" t="s">
+        <v>42</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C39" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A40" t="s">
+        <v>43</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C40" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A41" t="s">
+        <v>43</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C41" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A42" t="s">
+        <v>43</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C42" t="s">
+        <v>41</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Runtime fix, concentration parsing
Sometimes errored out when parsing concentrations, added a retry, and clarified the formatting.
</commit_message>
<xml_diff>
--- a/data/compound_library/library.xlsx
+++ b/data/compound_library/library.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10420"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10921"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/danbru/Library/CloudStorage/OneDrive-Chalmers/Desktop/GenExp/data/compound_library/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B706F176-FAFC-5E4A-A858-9609A912B726}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B48BA935-88AB-0F49-9BB9-BF74A08E2431}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-35840" yWindow="500" windowWidth="35840" windowHeight="21900" xr2:uid="{5207ED13-6406-E44B-8029-6CEF5067A94D}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="51200" windowHeight="27060" xr2:uid="{5207ED13-6406-E44B-8029-6CEF5067A94D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="46">
   <si>
     <t>Compound</t>
   </si>
@@ -597,7 +597,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C37B54C-13B4-4F49-B23D-63B14E507B7A}">
-  <dimension ref="A1:C42"/>
+  <dimension ref="A1:C50"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="28.33203125" customWidth="1"/>
@@ -640,13 +640,13 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="C4" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
@@ -657,7 +657,7 @@
         <v>8</v>
       </c>
       <c r="C5" t="s">
-        <v>13</v>
+        <v>25</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
@@ -668,7 +668,7 @@
         <v>8</v>
       </c>
       <c r="C6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
@@ -679,29 +679,29 @@
         <v>8</v>
       </c>
       <c r="C7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C8" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C9" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.2">
@@ -712,7 +712,7 @@
         <v>7</v>
       </c>
       <c r="C10" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.2">
@@ -723,7 +723,7 @@
         <v>7</v>
       </c>
       <c r="C11" t="s">
-        <v>14</v>
+        <v>25</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.2">
@@ -734,40 +734,40 @@
         <v>7</v>
       </c>
       <c r="C12" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="C13" t="s">
-        <v>25</v>
+        <v>14</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="C14" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="C15" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.2">
@@ -778,293 +778,381 @@
         <v>10</v>
       </c>
       <c r="C16" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="C17" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="C18" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="C19" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>24</v>
+        <v>10</v>
       </c>
       <c r="C20" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C21" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="C22" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="C23" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>26</v>
+        <v>5</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="C24" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>28</v>
+        <v>5</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="C25" t="s">
-        <v>13</v>
+        <v>25</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>28</v>
+        <v>11</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>29</v>
+        <v>12</v>
       </c>
       <c r="C26" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>31</v>
-      </c>
-      <c r="B27" s="4" t="s">
-        <v>30</v>
+        <v>11</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>12</v>
       </c>
       <c r="C27" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>31</v>
-      </c>
-      <c r="B28" s="4" t="s">
-        <v>30</v>
+        <v>26</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>27</v>
       </c>
       <c r="C28" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>31</v>
-      </c>
-      <c r="B29" s="4" t="s">
-        <v>30</v>
+        <v>26</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>27</v>
       </c>
       <c r="C29" t="s">
-        <v>32</v>
+        <v>19</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="C30" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="C31" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>33</v>
-      </c>
-      <c r="B32" s="2" t="s">
-        <v>34</v>
+        <v>31</v>
+      </c>
+      <c r="B32" s="4" t="s">
+        <v>30</v>
       </c>
       <c r="C32" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>33</v>
-      </c>
-      <c r="B33" s="2" t="s">
-        <v>34</v>
+        <v>31</v>
+      </c>
+      <c r="B33" s="4" t="s">
+        <v>30</v>
       </c>
       <c r="C33" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>35</v>
-      </c>
-      <c r="B34" s="2" t="s">
-        <v>39</v>
+        <v>31</v>
+      </c>
+      <c r="B34" s="4" t="s">
+        <v>30</v>
       </c>
       <c r="C34" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="C35" t="s">
-        <v>37</v>
+        <v>25</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="C36" t="s">
-        <v>38</v>
+        <v>13</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>42</v>
+        <v>33</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>45</v>
+        <v>34</v>
       </c>
       <c r="C37" t="s">
-        <v>40</v>
+        <v>14</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>42</v>
+        <v>33</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>45</v>
+        <v>34</v>
       </c>
       <c r="C38" t="s">
-        <v>36</v>
+        <v>15</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>42</v>
+        <v>33</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>45</v>
+        <v>34</v>
       </c>
       <c r="C39" t="s">
-        <v>41</v>
+        <v>19</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="C40" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="C41" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
+        <v>35</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C42" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A43" t="s">
+        <v>42</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C43" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A44" t="s">
+        <v>42</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C44" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A45" t="s">
+        <v>42</v>
+      </c>
+      <c r="B45" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C45" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A46" t="s">
+        <v>42</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C46" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A47" t="s">
         <v>43</v>
       </c>
-      <c r="B42" s="2" t="s">
+      <c r="B47" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="C42" t="s">
+      <c r="C47" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A48" t="s">
+        <v>43</v>
+      </c>
+      <c r="B48" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C48" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A49" t="s">
+        <v>43</v>
+      </c>
+      <c r="B49" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C49" t="s">
         <v>41</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A50" t="s">
+        <v>43</v>
+      </c>
+      <c r="B50" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C50" t="s">
+        <v>37</v>
       </c>
     </row>
   </sheetData>

</xml_diff>